<commit_message>
Add student management features and fix UI issues
</commit_message>
<xml_diff>
--- a/templates/results_template.xlsx
+++ b/templates/results_template.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SRMS\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4365896-7400-4962-ACCF-D22E82DD19E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Index No</t>
   </si>
@@ -35,62 +40,27 @@
     <t>Total Marks</t>
   </si>
   <si>
-    <t>IDX2025001</t>
-  </si>
-  <si>
-    <t>BR20250001</t>
-  </si>
-  <si>
     <t>CSE101</t>
   </si>
   <si>
     <t>Introduction to Programming</t>
   </si>
   <si>
-    <t>CSE102</t>
-  </si>
-  <si>
-    <t>Computer Fundamentals</t>
-  </si>
-  <si>
-    <t>IDX2025002</t>
-  </si>
-  <si>
-    <t>BR20250002</t>
-  </si>
-  <si>
-    <t>IDX2025003</t>
-  </si>
-  <si>
-    <t>BR20250003</t>
-  </si>
-  <si>
-    <t>EEE101</t>
-  </si>
-  <si>
-    <t>Basic Electrical</t>
+    <t>cst-m-1920</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -117,14 +87,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -414,22 +392,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="32.992" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -449,18 +423,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <v>759291</v>
+      </c>
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
       </c>
       <c r="E2">
         <v>85</v>
@@ -469,98 +443,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3">
-        <v>78</v>
-      </c>
-      <c r="F3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4">
-        <v>92</v>
-      </c>
-      <c r="F4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>88</v>
-      </c>
-      <c r="F5">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6">
-        <v>90</v>
-      </c>
-      <c r="F6">
-        <v>100</v>
-      </c>
-    </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>